<commit_message>
Remove Item Type column from PO entry and PO line register
Drops the column from the prototype sheets, the PO line blueprint and the
decision register; formulas re-pointed to the shifted columns. No columns added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014WLfSQhcddkfakQyHQVtKv
</commit_message>
<xml_diff>
--- a/prototype/1 ISKO Stores FY2027-28 (prototype).xlsx
+++ b/prototype/1 ISKO Stores FY2027-28 (prototype).xlsx
@@ -517,23 +517,22 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblPoLineRegister" displayName="tblPoLineRegister" ref="A4:N7" headerRowCount="1">
-  <autoFilter ref="A4:N7"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="tblPoLineRegister" displayName="tblPoLineRegister" ref="A4:M7" headerRowCount="1">
+  <autoFilter ref="A4:M7"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="PO Line ID"/>
     <tableColumn id="2" name="PO No"/>
-    <tableColumn id="3" name="Item Type"/>
-    <tableColumn id="4" name="Item ID"/>
-    <tableColumn id="5" name="Grade"/>
-    <tableColumn id="6" name="Thk mm"/>
-    <tableColumn id="7" name="L mm"/>
-    <tableColumn id="8" name="W mm"/>
-    <tableColumn id="9" name="Ordered kg"/>
-    <tableColumn id="10" name="Unit"/>
-    <tableColumn id="11" name="Rate Rs"/>
-    <tableColumn id="12" name="Line Value Rs"/>
-    <tableColumn id="13" name="Due Date"/>
-    <tableColumn id="14" name="Posted At"/>
+    <tableColumn id="3" name="Item ID"/>
+    <tableColumn id="4" name="Grade"/>
+    <tableColumn id="5" name="Thk mm"/>
+    <tableColumn id="6" name="L mm"/>
+    <tableColumn id="7" name="W mm"/>
+    <tableColumn id="8" name="Ordered kg"/>
+    <tableColumn id="9" name="Unit"/>
+    <tableColumn id="10" name="Rate Rs"/>
+    <tableColumn id="11" name="Line Value Rs"/>
+    <tableColumn id="12" name="Due Date"/>
+    <tableColumn id="13" name="Posted At"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showRowStripes="0"/>
 </table>
@@ -2714,11 +2713,11 @@
         <v/>
       </c>
       <c r="C5" s="22">
-        <f>INDEX('PO Line Register'!$D$5:$D$400,MATCH(A5,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$C$5:$C$400,MATCH(A5,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="D5" s="32">
-        <f>INDEX('PO Line Register'!$I$5:$I$400,MATCH(A5,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$H$5:$H$400,MATCH(A5,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="E5" s="30">
@@ -2730,7 +2729,7 @@
         <v/>
       </c>
       <c r="G5" s="37">
-        <f>INDEX('PO Line Register'!$M$5:$M$400,MATCH(A5,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$L$5:$L$400,MATCH(A5,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="H5" s="23">
@@ -2753,11 +2752,11 @@
         <v/>
       </c>
       <c r="C6" s="22">
-        <f>INDEX('PO Line Register'!$D$5:$D$400,MATCH(A6,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$C$5:$C$400,MATCH(A6,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="D6" s="32">
-        <f>INDEX('PO Line Register'!$I$5:$I$400,MATCH(A6,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$H$5:$H$400,MATCH(A6,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="E6" s="30">
@@ -2769,7 +2768,7 @@
         <v/>
       </c>
       <c r="G6" s="37">
-        <f>INDEX('PO Line Register'!$M$5:$M$400,MATCH(A6,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$L$5:$L$400,MATCH(A6,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="H6" s="23">
@@ -2792,11 +2791,11 @@
         <v/>
       </c>
       <c r="C7" s="22">
-        <f>INDEX('PO Line Register'!$D$5:$D$400,MATCH(A7,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$C$5:$C$400,MATCH(A7,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="D7" s="32">
-        <f>INDEX('PO Line Register'!$I$5:$I$400,MATCH(A7,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$H$5:$H$400,MATCH(A7,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="E7" s="30">
@@ -2808,7 +2807,7 @@
         <v/>
       </c>
       <c r="G7" s="37">
-        <f>INDEX('PO Line Register'!$M$5:$M$400,MATCH(A7,'PO Line Register'!$A$5:$A$400,0))</f>
+        <f>INDEX('PO Line Register'!$L$5:$L$400,MATCH(A7,'PO Line Register'!$A$5:$A$400,0))</f>
         <v/>
       </c>
       <c r="H7" s="23">
@@ -4007,23 +4006,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="30" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -4130,60 +4128,55 @@
       </c>
       <c r="C6" s="21" t="inlineStr">
         <is>
-          <t>Item Type</t>
+          <t>Item ID</t>
         </is>
       </c>
       <c r="D6" s="21" t="inlineStr">
         <is>
-          <t>Item ID</t>
+          <t>Grade</t>
         </is>
       </c>
       <c r="E6" s="21" t="inlineStr">
         <is>
-          <t>Grade</t>
+          <t>Thk mm</t>
         </is>
       </c>
       <c r="F6" s="21" t="inlineStr">
         <is>
-          <t>Thk mm</t>
+          <t>L mm</t>
         </is>
       </c>
       <c r="G6" s="21" t="inlineStr">
         <is>
-          <t>L mm</t>
+          <t>W mm</t>
         </is>
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
-          <t>W mm</t>
+          <t>Ordered kg</t>
         </is>
       </c>
       <c r="I6" s="21" t="inlineStr">
         <is>
-          <t>Ordered kg</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="J6" s="21" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Rate Rs</t>
         </is>
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
-          <t>Rate Rs</t>
+          <t>Line Value Rs</t>
         </is>
       </c>
       <c r="L6" s="21" t="inlineStr">
         <is>
-          <t>Line Value Rs</t>
+          <t>Due Date</t>
         </is>
       </c>
       <c r="M6" s="21" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="N6" s="21" t="inlineStr">
         <is>
           <t>Ready / issues</t>
         </is>
@@ -4194,52 +4187,47 @@
         <v>1</v>
       </c>
       <c r="B7" s="23">
-        <f>IF(D7="","",$B$3&amp;"-"&amp;TEXT(A7,"00"))</f>
+        <f>IF(C7="","",$B$3&amp;"-"&amp;TEXT(A7,"00"))</f>
         <v/>
       </c>
       <c r="C7" s="24" t="inlineStr">
         <is>
-          <t>RM</t>
-        </is>
-      </c>
-      <c r="D7" s="24" t="inlineStr">
-        <is>
           <t>GPSP-1.6</t>
         </is>
       </c>
+      <c r="D7" s="23">
+        <f>IF(C7="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(C7,'M_Material'!$A$5:$A$50,0)),"?"))</f>
+        <v/>
+      </c>
       <c r="E7" s="23">
-        <f>IF(D7="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(D7,'M_Material'!$A$5:$A$50,0)),"?"))</f>
-        <v/>
-      </c>
-      <c r="F7" s="23">
-        <f>IF(D7="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(D7,'M_Material'!$A$5:$A$50,0)),""))</f>
-        <v/>
+        <f>IF(C7="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(C7,'M_Material'!$A$5:$A$50,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F7" s="24" t="n">
+        <v>2500</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H7" s="24" t="n">
         <v>1250</v>
       </c>
-      <c r="I7" s="25" t="n">
+      <c r="H7" s="25" t="n">
         <v>2000</v>
       </c>
-      <c r="J7" s="23">
-        <f>IF(D7="","","KGS")</f>
-        <v/>
-      </c>
-      <c r="K7" s="26" t="n">
+      <c r="I7" s="23">
+        <f>IF(C7="","","KGS")</f>
+        <v/>
+      </c>
+      <c r="J7" s="26" t="n">
         <v>74.5</v>
       </c>
-      <c r="L7" s="27">
-        <f>IF(I7="","",ROUND(I7*K7,2))</f>
-        <v/>
-      </c>
-      <c r="M7" s="28" t="n">
+      <c r="K7" s="27">
+        <f>IF(H7="","",ROUND(H7*J7,2))</f>
+        <v/>
+      </c>
+      <c r="L7" s="28" t="n">
         <v>46502</v>
       </c>
-      <c r="N7" s="29">
-        <f>IF(D7="","",IF(E7="?","ITEM NOT IN MASTER",IF(N(I7)&lt;=0,"QTY REQUIRED",IF(N(K7)&lt;=0,"RATE REQUIRED",IF(M7&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
+      <c r="M7" s="29">
+        <f>IF(C7="","",IF(D7="?","ITEM NOT IN MASTER",IF(N(H7)&lt;=0,"QTY REQUIRED",IF(N(J7)&lt;=0,"RATE REQUIRED",IF(L7&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
         <v/>
       </c>
     </row>
@@ -4248,50 +4236,45 @@
         <v>2</v>
       </c>
       <c r="B8" s="23">
-        <f>IF(D8="","",$B$3&amp;"-"&amp;TEXT(A8,"00"))</f>
+        <f>IF(C8="","",$B$3&amp;"-"&amp;TEXT(A8,"00"))</f>
         <v/>
       </c>
       <c r="C8" s="24" t="inlineStr">
         <is>
-          <t>RM</t>
-        </is>
-      </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
           <t>HRCA-2.0</t>
         </is>
       </c>
+      <c r="D8" s="23">
+        <f>IF(C8="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(C8,'M_Material'!$A$5:$A$50,0)),"?"))</f>
+        <v/>
+      </c>
       <c r="E8" s="23">
-        <f>IF(D8="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(D8,'M_Material'!$A$5:$A$50,0)),"?"))</f>
-        <v/>
-      </c>
-      <c r="F8" s="23">
-        <f>IF(D8="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(D8,'M_Material'!$A$5:$A$50,0)),""))</f>
-        <v/>
+        <f>IF(C8="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(C8,'M_Material'!$A$5:$A$50,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F8" s="24" t="n">
+        <v>2500</v>
       </c>
       <c r="G8" s="24" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H8" s="24" t="n">
         <v>1250</v>
       </c>
-      <c r="I8" s="25" t="n">
+      <c r="H8" s="25" t="n">
         <v>800</v>
       </c>
-      <c r="J8" s="23">
-        <f>IF(D8="","","KGS")</f>
-        <v/>
-      </c>
-      <c r="K8" s="26" t="n"/>
-      <c r="L8" s="27">
-        <f>IF(I8="","",ROUND(I8*K8,2))</f>
-        <v/>
-      </c>
-      <c r="M8" s="28" t="n">
+      <c r="I8" s="23">
+        <f>IF(C8="","","KGS")</f>
+        <v/>
+      </c>
+      <c r="J8" s="26" t="n"/>
+      <c r="K8" s="27">
+        <f>IF(H8="","",ROUND(H8*J8,2))</f>
+        <v/>
+      </c>
+      <c r="L8" s="28" t="n">
         <v>46502</v>
       </c>
-      <c r="N8" s="29">
-        <f>IF(D8="","",IF(E8="?","ITEM NOT IN MASTER",IF(N(I8)&lt;=0,"QTY REQUIRED",IF(N(K8)&lt;=0,"RATE REQUIRED",IF(M8&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
+      <c r="M8" s="29">
+        <f>IF(C8="","",IF(D8="?","ITEM NOT IN MASTER",IF(N(H8)&lt;=0,"QTY REQUIRED",IF(N(J8)&lt;=0,"RATE REQUIRED",IF(L8&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
         <v/>
       </c>
     </row>
@@ -4300,52 +4283,47 @@
         <v>3</v>
       </c>
       <c r="B9" s="23">
-        <f>IF(D9="","",$B$3&amp;"-"&amp;TEXT(A9,"00"))</f>
+        <f>IF(C9="","",$B$3&amp;"-"&amp;TEXT(A9,"00"))</f>
         <v/>
       </c>
       <c r="C9" s="24" t="inlineStr">
         <is>
-          <t>RM</t>
-        </is>
-      </c>
-      <c r="D9" s="24" t="inlineStr">
-        <is>
           <t>GPSP-2.5</t>
         </is>
       </c>
+      <c r="D9" s="23">
+        <f>IF(C9="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(C9,'M_Material'!$A$5:$A$50,0)),"?"))</f>
+        <v/>
+      </c>
       <c r="E9" s="23">
-        <f>IF(D9="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(D9,'M_Material'!$A$5:$A$50,0)),"?"))</f>
-        <v/>
-      </c>
-      <c r="F9" s="23">
-        <f>IF(D9="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(D9,'M_Material'!$A$5:$A$50,0)),""))</f>
-        <v/>
+        <f>IF(C9="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(C9,'M_Material'!$A$5:$A$50,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F9" s="24" t="n">
+        <v>2500</v>
       </c>
       <c r="G9" s="24" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H9" s="24" t="n">
         <v>1250</v>
       </c>
-      <c r="I9" s="25" t="n">
+      <c r="H9" s="25" t="n">
         <v>500</v>
       </c>
-      <c r="J9" s="23">
-        <f>IF(D9="","","KGS")</f>
-        <v/>
-      </c>
-      <c r="K9" s="26" t="n">
+      <c r="I9" s="23">
+        <f>IF(C9="","","KGS")</f>
+        <v/>
+      </c>
+      <c r="J9" s="26" t="n">
         <v>75</v>
       </c>
-      <c r="L9" s="27">
-        <f>IF(I9="","",ROUND(I9*K9,2))</f>
-        <v/>
-      </c>
-      <c r="M9" s="28" t="n">
+      <c r="K9" s="27">
+        <f>IF(H9="","",ROUND(H9*J9,2))</f>
+        <v/>
+      </c>
+      <c r="L9" s="28" t="n">
         <v>46502</v>
       </c>
-      <c r="N9" s="29">
-        <f>IF(D9="","",IF(E9="?","ITEM NOT IN MASTER",IF(N(I9)&lt;=0,"QTY REQUIRED",IF(N(K9)&lt;=0,"RATE REQUIRED",IF(M9&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
+      <c r="M9" s="29">
+        <f>IF(C9="","",IF(D9="?","ITEM NOT IN MASTER",IF(N(H9)&lt;=0,"QTY REQUIRED",IF(N(J9)&lt;=0,"RATE REQUIRED",IF(L9&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
         <v/>
       </c>
     </row>
@@ -4354,65 +4332,60 @@
         <v>4</v>
       </c>
       <c r="B10" s="23">
-        <f>IF(D10="","",$B$3&amp;"-"&amp;TEXT(A10,"00"))</f>
+        <f>IF(C10="","",$B$3&amp;"-"&amp;TEXT(A10,"00"))</f>
         <v/>
       </c>
       <c r="C10" s="24" t="inlineStr">
         <is>
-          <t>RM</t>
-        </is>
-      </c>
-      <c r="D10" s="24" t="inlineStr">
-        <is>
           <t>CRCA-1.0</t>
         </is>
       </c>
+      <c r="D10" s="23">
+        <f>IF(C10="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(C10,'M_Material'!$A$5:$A$50,0)),"?"))</f>
+        <v/>
+      </c>
       <c r="E10" s="23">
-        <f>IF(D10="","",IFERROR(INDEX('M_Material'!$C$5:$C$50,MATCH(D10,'M_Material'!$A$5:$A$50,0)),"?"))</f>
-        <v/>
-      </c>
-      <c r="F10" s="23">
-        <f>IF(D10="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(D10,'M_Material'!$A$5:$A$50,0)),""))</f>
-        <v/>
+        <f>IF(C10="","",IFERROR(INDEX('M_Material'!$D$5:$D$50,MATCH(C10,'M_Material'!$A$5:$A$50,0)),""))</f>
+        <v/>
+      </c>
+      <c r="F10" s="24" t="n">
+        <v>2500</v>
       </c>
       <c r="G10" s="24" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H10" s="24" t="n">
         <v>1250</v>
       </c>
-      <c r="I10" s="25" t="n">
+      <c r="H10" s="25" t="n">
         <v>1000</v>
       </c>
-      <c r="J10" s="23">
-        <f>IF(D10="","","KGS")</f>
-        <v/>
-      </c>
-      <c r="K10" s="26" t="n">
+      <c r="I10" s="23">
+        <f>IF(C10="","","KGS")</f>
+        <v/>
+      </c>
+      <c r="J10" s="26" t="n">
         <v>68.2</v>
       </c>
-      <c r="L10" s="27">
-        <f>IF(I10="","",ROUND(I10*K10,2))</f>
-        <v/>
-      </c>
-      <c r="M10" s="28" t="n">
+      <c r="K10" s="27">
+        <f>IF(H10="","",ROUND(H10*J10,2))</f>
+        <v/>
+      </c>
+      <c r="L10" s="28" t="n">
         <v>46478</v>
       </c>
-      <c r="N10" s="29">
-        <f>IF(D10="","",IF(E10="?","ITEM NOT IN MASTER",IF(N(I10)&lt;=0,"QTY REQUIRED",IF(N(K10)&lt;=0,"RATE REQUIRED",IF(M10&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
+      <c r="M10" s="29">
+        <f>IF(C10="","",IF(D10="?","ITEM NOT IN MASTER",IF(N(H10)&lt;=0,"QTY REQUIRED",IF(N(J10)&lt;=0,"RATE REQUIRED",IF(L10&lt;$B$4,"WARN: DUE BEFORE PO DATE","READY")))))</f>
         <v/>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="N7:N10">
+  <conditionalFormatting sqref="M7:M10">
     <cfRule type="expression" priority="1" dxfId="0" stopIfTrue="1">
-      <formula>OR(LEFT(N7,5)="READY",N7="OK",LEFT(N7,6)="CLOSED")</formula>
+      <formula>OR(LEFT(M7,5)="READY",M7="OK",LEFT(M7,6)="CLOSED")</formula>
     </cfRule>
     <cfRule type="expression" priority="2" dxfId="1" stopIfTrue="1">
-      <formula>OR(LEFT(N7,4)="WARN",LEFT(N7,2)="IN",LEFT(N7,3)="NOT",LEFT(N7,7)="REORDER",LEFT(N7,5)="STALE",LEFT(N7,4)="PART",LEFT(N7,7)="PENDING",LEFT(N7,5)="READY")</formula>
+      <formula>OR(LEFT(M7,4)="WARN",LEFT(M7,2)="IN",LEFT(M7,3)="NOT",LEFT(M7,7)="REORDER",LEFT(M7,5)="STALE",LEFT(M7,4)="PART",LEFT(M7,7)="PENDING",LEFT(M7,5)="READY")</formula>
     </cfRule>
     <cfRule type="expression" priority="3" dxfId="2">
-      <formula>LEN(N7)&gt;0</formula>
+      <formula>LEN(M7)&gt;0</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6201,7 +6174,7 @@
         </is>
       </c>
       <c r="F5" s="23">
-        <f>IF(E5="","",IFERROR(INDEX('PO Line Register'!$D$5:$D$400,MATCH(E5,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E5="","",IFERROR(INDEX('PO Line Register'!$C$5:$C$400,MATCH(E5,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="G5" s="23">
@@ -6241,7 +6214,7 @@
         <v>74.5</v>
       </c>
       <c r="Q5" s="27">
-        <f>IF(E5="","",IFERROR(INDEX('PO Line Register'!$K$5:$K$400,MATCH(E5,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E5="","",IFERROR(INDEX('PO Line Register'!$J$5:$J$400,MATCH(E5,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="R5" s="32">
@@ -6281,7 +6254,7 @@
         </is>
       </c>
       <c r="F6" s="23">
-        <f>IF(E6="","",IFERROR(INDEX('PO Line Register'!$D$5:$D$400,MATCH(E6,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E6="","",IFERROR(INDEX('PO Line Register'!$C$5:$C$400,MATCH(E6,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="G6" s="23">
@@ -6321,7 +6294,7 @@
         <v>74.5</v>
       </c>
       <c r="Q6" s="27">
-        <f>IF(E6="","",IFERROR(INDEX('PO Line Register'!$K$5:$K$400,MATCH(E6,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E6="","",IFERROR(INDEX('PO Line Register'!$J$5:$J$400,MATCH(E6,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="R6" s="32">
@@ -6361,7 +6334,7 @@
         </is>
       </c>
       <c r="F7" s="23">
-        <f>IF(E7="","",IFERROR(INDEX('PO Line Register'!$D$5:$D$400,MATCH(E7,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E7="","",IFERROR(INDEX('PO Line Register'!$C$5:$C$400,MATCH(E7,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="G7" s="23">
@@ -6401,7 +6374,7 @@
         <v>68.2</v>
       </c>
       <c r="Q7" s="27">
-        <f>IF(E7="","",IFERROR(INDEX('PO Line Register'!$K$5:$K$400,MATCH(E7,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E7="","",IFERROR(INDEX('PO Line Register'!$J$5:$J$400,MATCH(E7,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="R7" s="32">
@@ -6437,7 +6410,7 @@
         </is>
       </c>
       <c r="F8" s="23">
-        <f>IF(E8="","",IFERROR(INDEX('PO Line Register'!$D$5:$D$400,MATCH(E8,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E8="","",IFERROR(INDEX('PO Line Register'!$C$5:$C$400,MATCH(E8,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="G8" s="23">
@@ -6477,7 +6450,7 @@
         <v>68.2</v>
       </c>
       <c r="Q8" s="27">
-        <f>IF(E8="","",IFERROR(INDEX('PO Line Register'!$K$5:$K$400,MATCH(E8,'PO Line Register'!$A$5:$A$400,0)),""))</f>
+        <f>IF(E8="","",IFERROR(INDEX('PO Line Register'!$J$5:$J$400,MATCH(E8,'PO Line Register'!$A$5:$A$400,0)),""))</f>
         <v/>
       </c>
       <c r="R8" s="32">
@@ -8075,23 +8048,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N7"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="8" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
     <col width="7" customWidth="1" min="5" max="5"/>
     <col width="7" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
-    <col width="7" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="6" customWidth="1" min="10" max="10"/>
-    <col width="8" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="6" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="13" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -8121,60 +8093,55 @@
       </c>
       <c r="C4" s="21" t="inlineStr">
         <is>
-          <t>Item Type</t>
+          <t>Item ID</t>
         </is>
       </c>
       <c r="D4" s="21" t="inlineStr">
         <is>
-          <t>Item ID</t>
+          <t>Grade</t>
         </is>
       </c>
       <c r="E4" s="21" t="inlineStr">
         <is>
-          <t>Grade</t>
+          <t>Thk mm</t>
         </is>
       </c>
       <c r="F4" s="21" t="inlineStr">
         <is>
-          <t>Thk mm</t>
+          <t>L mm</t>
         </is>
       </c>
       <c r="G4" s="21" t="inlineStr">
         <is>
-          <t>L mm</t>
+          <t>W mm</t>
         </is>
       </c>
       <c r="H4" s="21" t="inlineStr">
         <is>
-          <t>W mm</t>
+          <t>Ordered kg</t>
         </is>
       </c>
       <c r="I4" s="21" t="inlineStr">
         <is>
-          <t>Ordered kg</t>
+          <t>Unit</t>
         </is>
       </c>
       <c r="J4" s="21" t="inlineStr">
         <is>
-          <t>Unit</t>
+          <t>Rate Rs</t>
         </is>
       </c>
       <c r="K4" s="21" t="inlineStr">
         <is>
-          <t>Rate Rs</t>
+          <t>Line Value Rs</t>
         </is>
       </c>
       <c r="L4" s="21" t="inlineStr">
         <is>
-          <t>Line Value Rs</t>
+          <t>Due Date</t>
         </is>
       </c>
       <c r="M4" s="21" t="inlineStr">
-        <is>
-          <t>Due Date</t>
-        </is>
-      </c>
-      <c r="N4" s="21" t="inlineStr">
         <is>
           <t>Posted At</t>
         </is>
@@ -8193,46 +8160,41 @@
       </c>
       <c r="C5" s="23" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>GPSP-1.6</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>GPSP-1.6</t>
-        </is>
-      </c>
-      <c r="E5" s="23" t="inlineStr">
-        <is>
           <t>GPSP</t>
         </is>
       </c>
+      <c r="E5" s="23" t="n">
+        <v>1.6</v>
+      </c>
       <c r="F5" s="23" t="n">
-        <v>1.6</v>
+        <v>2500</v>
       </c>
       <c r="G5" s="23" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H5" s="23" t="n">
         <v>1250</v>
       </c>
-      <c r="I5" s="30" t="n">
+      <c r="H5" s="30" t="n">
         <v>3000</v>
       </c>
-      <c r="J5" s="23" t="inlineStr">
+      <c r="I5" s="23" t="inlineStr">
         <is>
           <t>KGS</t>
         </is>
       </c>
+      <c r="J5" s="27" t="n">
+        <v>74.5</v>
+      </c>
       <c r="K5" s="27" t="n">
-        <v>74.5</v>
-      </c>
-      <c r="L5" s="27" t="n">
         <v>223500</v>
       </c>
-      <c r="M5" s="35" t="n">
+      <c r="L5" s="35" t="n">
         <v>46489</v>
       </c>
-      <c r="N5" s="36" t="n">
+      <c r="M5" s="36" t="n">
         <v>46479.46180555555</v>
       </c>
     </row>
@@ -8249,46 +8211,41 @@
       </c>
       <c r="C6" s="23" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>GPSP-1.2</t>
         </is>
       </c>
       <c r="D6" s="23" t="inlineStr">
         <is>
-          <t>GPSP-1.2</t>
-        </is>
-      </c>
-      <c r="E6" s="23" t="inlineStr">
-        <is>
           <t>GPSP</t>
         </is>
       </c>
+      <c r="E6" s="23" t="n">
+        <v>1.2</v>
+      </c>
       <c r="F6" s="23" t="n">
-        <v>1.2</v>
+        <v>2500</v>
       </c>
       <c r="G6" s="23" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H6" s="23" t="n">
         <v>1250</v>
       </c>
-      <c r="I6" s="30" t="n">
+      <c r="H6" s="30" t="n">
         <v>2400</v>
       </c>
-      <c r="J6" s="23" t="inlineStr">
+      <c r="I6" s="23" t="inlineStr">
         <is>
           <t>KGS</t>
         </is>
       </c>
+      <c r="J6" s="27" t="n">
+        <v>74.5</v>
+      </c>
       <c r="K6" s="27" t="n">
-        <v>74.5</v>
-      </c>
-      <c r="L6" s="27" t="n">
         <v>178800</v>
       </c>
-      <c r="M6" s="35" t="n">
+      <c r="L6" s="35" t="n">
         <v>46489</v>
       </c>
-      <c r="N6" s="36" t="n">
+      <c r="M6" s="36" t="n">
         <v>46479.46180555555</v>
       </c>
     </row>
@@ -8305,46 +8262,41 @@
       </c>
       <c r="C7" s="23" t="inlineStr">
         <is>
-          <t>RM</t>
+          <t>CRCA-1.0</t>
         </is>
       </c>
       <c r="D7" s="23" t="inlineStr">
         <is>
-          <t>CRCA-1.0</t>
-        </is>
-      </c>
-      <c r="E7" s="23" t="inlineStr">
-        <is>
           <t>CRCA</t>
         </is>
       </c>
+      <c r="E7" s="23" t="n">
+        <v>1</v>
+      </c>
       <c r="F7" s="23" t="n">
-        <v>1</v>
+        <v>2500</v>
       </c>
       <c r="G7" s="23" t="n">
-        <v>2500</v>
-      </c>
-      <c r="H7" s="23" t="n">
         <v>1250</v>
       </c>
-      <c r="I7" s="30" t="n">
+      <c r="H7" s="30" t="n">
         <v>1500</v>
       </c>
-      <c r="J7" s="23" t="inlineStr">
+      <c r="I7" s="23" t="inlineStr">
         <is>
           <t>KGS</t>
         </is>
       </c>
+      <c r="J7" s="27" t="n">
+        <v>68.2</v>
+      </c>
       <c r="K7" s="27" t="n">
-        <v>68.2</v>
-      </c>
-      <c r="L7" s="27" t="n">
         <v>102300</v>
       </c>
-      <c r="M7" s="35" t="n">
+      <c r="L7" s="35" t="n">
         <v>46491</v>
       </c>
-      <c r="N7" s="36" t="n">
+      <c r="M7" s="36" t="n">
         <v>46480.69444444445</v>
       </c>
     </row>

</xml_diff>